<commit_message>
Automatiza 11 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG POWERADE MOD 1.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG POWERADE MOD 1.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Plan1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -341,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -608,6 +608,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PG POWERADE MOD 1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ESTRUTURA TUBULAR CORPO LARGO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>98</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>002027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>